<commit_message>
Spec: RUNBOOK-48 Part D — 6 stakeholder-added business questions (T22-T27)
Add the leader's review questions as a distinct cross-tool Q&A block,
reviewed from Codex's internal-box draft:
- T22 MDC table count (capability boundary: no read-only DB-catalog tool)
- T23 use-case counts HASE/non-HASE (source_system_impact + UAT snapshot)
- T24 SMS feedback-status repos (term disambiguation)
- T25 PN opt-in logic + repos (deep logic)
- T26 2-way SMS repos (message graph)
- T27 WeChat channel type (official account, not personal/WeCom)

Excel: rows 25-30 in 全工具冒烟 sheet, smoke stats kept scoped to T1-T21.
Runbook: new Part D table + Send-back checklist; noted these don't change
the 21-tool coverage invariant. Added T23 caliber caveat (MDC-as-platform
vs source_system field value).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RUNBOOK-48-test-questions.xlsx
+++ b/RUNBOOK-48-test-questions.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1610,6 +1610,270 @@
         </is>
       </c>
     </row>
+    <row r="25" ht="62" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>T22</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>DB catalog(当前无工具)</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ 能力边界</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>MDC 的数据库现在一共有多少张表？</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>应查询 live DB 的只读 catalog/schema(当前工具集里没有这个工具);现阶段只能辅助检查 UAT snapshot manifest + 离线数据库设计摘录</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>当前无法权威回答 live MDC database 的表总数,不能猜。可证明的只有:1) UAT snapshot 20260720-1730 实际导出 3 张表:tbl_use_case(2,810 行)、tbl_use_case_channel_rule(6,217 行)、tbl_use_case_ext(2,660 行);2) 离线数据库设计摘录列出 8 张 use-case 相关表。「导出 3 张」和「设计列 8 张」都≠整个 live MDC DB 的表总数。要真实答案须 DBA 提供只读 schema/catalog 导出(如 information_schema.tables 结果)或开放只读 DB catalog 工具。</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>禁止把 UAT 快照的 3 张表、设计文档的 8 张表、或 Java @Table 类数量冒充 live DB 总表数。证据:index/usecase-snapshots/uat/20260720-1730/manifest.json;.tmp/use_case_db_design_tables.md</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="n"/>
+      <c r="I25" s="5" t="n"/>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>待测</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="62" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>source_system_impact + UAT snapshot</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ 口径边界</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>MDC 现在有多少 use cases？HASE 和 non-HASE 各多少？</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>source_system_impact(source_system="MDC") + 对 UAT tbl_use_case.snapshot.csv 按 group_member 统计(source_system 大小写归一)</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>按 UAT snapshot 20260720-1730 的 total 口径:MDC 共 880 个 use cases;HASE 819;non-HASE 61。non-HASE 的 61 = HSBC 56 + group_member 空白/未知 5,不能把这 5 条未填写记录静默算成 HSBC。若只数当前 active:总数 876;HASE 817;non-HASE 59(HSBC 56 + 空白/未知 3);另有 inactive 4。回答必须同时写明 snapshot 时间与 total/active 口径。★口径说明:此处「MDC」按整个消息平台(tbl_use_case 全量)理解,用 source_system_impact(source_system="MDC") 取平台总数;若把 MDC 当成 source_system 字段值之一(MDC/PEGA/eAlert…)则数字含义不同——回答须说明用的是哪一种读法。</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>source_system_impact 可直接证明 MDC total=880、active=876、inactive=4;HASE/HSBC/空白拆分来自 UAT tbl_use_case 正式字段 group_member。证据:index/usecase-snapshots/uat/20260720-1730/tbl_use_case.snapshot.csv;.tmp/use_case_db_design_tables.md(group_member 示例值 HASE)</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="n"/>
+      <c r="I26" s="5" t="n"/>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>待测</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="62" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>T24</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>list_repos + search_code/read_file</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ 术语消歧</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>请列出与 SMS feedback status 相关的 repo。</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>list_repos(query="feedback") + list_repos(query="tracking") + list_repos(channel="sms") + scoped search_code/read_file</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>必须先澄清「feedback status」含义:A. 若指客户点击/行为反馈:名称检索到 mc-hk-hase-email-feedback-api、mc-hk-hase-feedback-api、mc-hk-hase-wsb-feedback-api,但代码显示它们分别偏 Email、In-app/Push、WSB In-app,并非 SMS 投递回执主链。B. 若指 SMS 发送/投递状态(更贴合本题):核心 repos 应分层列出——状态 API:mc-hk-hase-htcl-tracking-api、amet-mdc-hsbc-cm-tracking-api;共享调用/配置:mc-hk-hase-api-rest-invoker、mc-hk-hase-api-starter;实际 tracking jobs:mc-hk-hase-svc-rt-gen-tracking-job、mc-hk-hase-svc-bat-tracking-job、mc-hk-hase-ssvc-bat-tracking-job。不能把搜到的全部 36 个 tracking 或 70 个 SMS 仓库不加区分当答案。</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>成功证据应含真实接口/配置:HTCL /v4/query-sms-status(含 /otp);CM POST /api/sms-status;api-starter 的 querySmsStatus 下游 URL;tracking job 里 Htcl/Csl/Cm/Lx SMS tracker 类。代码位置示例:mirror/mc-hk-hase-api-starter/src/main/resources/application-downstream-prod.yaml:256-286;CmStatusTrackingResource.java:29</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="n"/>
+      <c r="I27" s="5" t="n"/>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>待测</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="62" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>T25</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>list_repos + search_code/read_file</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ 深度逻辑</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>需要检查 PN 的 opt-in status;请给出 repo 并总结 Push Notification opt-in 逻辑。</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>list_repos(query="preference") + scoped search_code(PushMessageValidator/AlertTypeEnum/PreferenceResource) + read_file</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>「opin」按上下文应理解为 opt-in。核心 repos:Preference 入口/资料维护:mc-hk-hase-preferences-api、mc-hk-hase-preferences-job;发送前把关:mc-hk-hase-api-dispatch-core、mc-hk-hase-api-delivery-core;共享支持:mc-hk-hase-api-rest-invoker、mc-hk-hase-api-common、mc-hk-hase-api-domain。逻辑:1) verifyPushPoint=false 时跳过检查;2) 必须找到客户资料;3) 必须有 device token,delivery-core 还把「NA」视为无 token;4) 必须有 Use Case 配置和客户 subscription list;5) Use Case 哪个 Push opt-in flag 为 Y,就必须在客户 subscription 找到同一 alertType 且 alertChannelStatus03=Y;6) 不满足即抛 NotOptInException 阻止继续发送。覆盖普通、高风险、Marketing、Credit Card 00507、Investment 99998、Securities 等 Push;delivery-core 还含 Marketing Insight。注意:opt-in 只证明「允许/有资格发送」,不证明消息实际已送达。</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>关键证据:preferences-api PreferenceResource.java:38-62;preferences-job DaascProcessService.java:133-145,256-332;api-dispatch-core PushMessageValidator.java:30-119;api-delivery-core PushMessageValidator.java:33-128;rest-invoker 的 CreatePnPreferenceInvoker(POST)/UpdatePnPreferenceInvoker(PUT)</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="n"/>
+      <c r="I28" s="5" t="n"/>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>待测</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="62" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>T26</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>list_repos + 消息图(producers/consumers)</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>🟢 消息图</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>请列出与 2-way SMS 相关的 repo。</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>list_repos(query="2way") + producers/consumers(destination="hrn.hase.shared.notification.2way_sms_reply") + repo_routes + scoped source search</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>不能只回答名称里带 2way 的那 1 个仓库;完整主链按职责列出——发出 2-way SMS:mc-hk-hase-svc-rt-hr-htcl-2way-sms-deli-job;接收客户回复:mc-hk-hase-hutchison-inbound-gateway;消费回复/对账报表:mc-hk-hase-reconciliation-report-job;查询投递状态:mc-hk-hase-svc-rt-hr-tracking-job(含 Htcl2WaySmsTracker / Htcl2WaySmsPollTracker);共享业务库:mc-hk-hase-api-delivery-core、mc-hk-hase-api-tracking-core、mc-hk-hase-api-dao、mc-hk-hase-api-domain、mc-hk-hase-api-rest-invoker(含 ReplyFraudFeedbackInvoker)。</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>消息图证据:reply topic「hrn.hase.shared.notification.2way_sms_reply」的 producer=mc-hk-hase-hutchison-inbound-gateway、consumer=mc-hk-hase-reconciliation-report-job(index/message_edges.csv:206);outbound delivery topic 边在 index/message_edges.csv:385。list_repos(query="2way") 只返回 1 个命名撞中的仓库,不代表主链只有 1 个 repo。</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="n"/>
+      <c r="I29" s="5" t="n"/>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>待测</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="62" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>T27</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>list_repos + repo_routes + search_code</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ 渠道边界</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>WeChat 用的是 personal chat channel 还是 company WeChat channel？</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>list_repos(channel="wechat") + repo_routes + scoped search_code(openid/template_id/corpId/agentId/qyapi.weixin.qq.com)</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>现有代码最符合「腾讯微信公众号(Official Account)」模板消息,不是个人对个人的 peer-to-peer chat;同时也没有证据表明是企业微信/WeCom。证据特征:按用户 openid 发送、用 appid/appsecret + access token、调 /cgi-bin/message/template/send、请求体字段 touser/template_id/data。相关 delivery repos 只有 2 个:mc-hk-hase-ssvc-rt-gen-wechat-deli-job(realtime general)、mc-hk-hase-ssvc-rt-hr-wechat-deli-job(realtime high-risk),两者差异是 general/high-risk,不是 personal/company。代码里未见企业微信常见的 corpId、agentId 或 qyapi.weixin.qq.com。</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>关键证据:api-starter application-downstream.yaml:591-595;SendWeChatMessageRequest.java:29-33;WeChatService.java:86-125;TencentWechatRouter.java:54-84,110-133。回答时别把「向个人 openid 发公众号消息」误写成「个人聊天」,也别把公众号误写成企业微信。</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="n"/>
+      <c r="I30" s="5" t="n"/>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>待测</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1622,7 +1886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1694,22 +1958,33 @@
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>已判定 PASS</t>
+          <t>已判定 PASS(含 T22–T27)</t>
         </is>
       </c>
       <c r="B8" s="11">
-        <f>COUNTIF(全工具冒烟!J2:J24,"PASS")</f>
+        <f>COUNTIF(全工具冒烟!J2:J30,"PASS")</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>已判定 FAIL</t>
+          <t>已判定 FAIL(含 T22–T27)</t>
         </is>
       </c>
       <c r="B9" s="11">
-        <f>COUNTIF(全工具冒烟!J2:J24,"FAIL")</f>
+        <f>COUNTIF(全工具冒烟!J2:J30,"FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>领导追加业务问题(T22–T27,跨工具 Q&amp;A)</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>COUNTA(全工具冒烟!A25:A30)</f>
         <v/>
       </c>
     </row>
@@ -1759,6 +2034,13 @@
       <c r="A18" s="13" t="inlineStr">
         <is>
           <t>6. K3002 是 Codex 实测可用的固定 use_case_id(同时在 UAT 主数据和 dev/SCT 快照里,能覆盖 rule_text AST);&lt;完整topic&gt;/&lt;未索引仓库的类&gt; 这类占位内网用真实数据替换,找靶子步骤见 runbook Part B(用 manifest 的 staged_repos,备选靶子 SapiAutoScanConfig)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>7. T22–T27 是业务方/领导会议追加的跨工具业务问题(不是单工具冒烟):T22 测「没有只读 DB catalog 工具」的能力边界,T23 走 source_system_impact + UAT 快照口径,T24–T27 组合 list_repos / search_code / read_file / 消息图 / repo_routes。类型标签(能力边界/口径边界/术语消歧/深度逻辑/消息图/渠道边界)是问题类别,不是冒烟图例;它们不影响 runbook Part C 的 21==21 工具覆盖不变量。</t>
         </is>
       </c>
     </row>

</xml_diff>